<commit_message>
Rekonsiliasi: tanggal blok tanpa-tanggal (A2609302102 Batam Sortation + A2610080552) diputuskan 12 Okt 2026 berdasarkan hasil cek Supabase (DB lama 11 Okt = 12 kena bug -1 hari) — regenerasi file upload-ulang 13 OKT, Excel, expected-lines, dan SQL CEK; SQL PERBAIKI tidak berubah
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/rekonsiliasi/HASIL-COCOKAN-12-15-OKT-2026.xlsx
+++ b/rekonsiliasi/HASIL-COCOKAN-12-15-OKT-2026.xlsx
@@ -790,31 +790,31 @@
         <v>2026-10-12</v>
       </c>
       <c r="B3" t="str">
-        <v>A2610050285</v>
+        <v>A2609302102</v>
       </c>
       <c r="C3" t="str">
-        <v>SiCepat Ekspres Medan Sortation</v>
+        <v>SiCepat Ekspres Batam Sortation</v>
       </c>
       <c r="D3" t="str">
-        <v>201025</v>
+        <v>502004</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F3">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="J3" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="4">
@@ -822,19 +822,19 @@
         <v>2026-10-12</v>
       </c>
       <c r="B4" t="str">
-        <v>A2610080518</v>
+        <v>A2610050285</v>
       </c>
       <c r="C4" t="str">
-        <v>SiCepat Ekspres Jombang Sortation</v>
+        <v>SiCepat Ekspres Medan Sortation</v>
       </c>
       <c r="D4" t="str">
-        <v>1618003</v>
+        <v>201025</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -843,7 +843,7 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J4" t="str">
         <v>12 OKT</v>
@@ -854,19 +854,19 @@
         <v>2026-10-12</v>
       </c>
       <c r="B5" t="str">
-        <v>A2610100732</v>
+        <v>A2610080518</v>
       </c>
       <c r="C5" t="str">
-        <v>SiCepat Ekspres Cikarang Utara FM</v>
+        <v>SiCepat Ekspres Jombang Sortation</v>
       </c>
       <c r="D5" t="str">
-        <v>1209094</v>
+        <v>1618003</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -875,7 +875,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J5" t="str">
         <v>12 OKT</v>
@@ -886,31 +886,31 @@
         <v>2026-10-12</v>
       </c>
       <c r="B6" t="str">
-        <v>A2610110733</v>
+        <v>A2610080552</v>
       </c>
       <c r="C6" t="str">
-        <v>SiCepat Ekspres Jakut Penjaringan 2 FM</v>
+        <v>Jakbar Kalideres FM</v>
       </c>
       <c r="D6" t="str">
-        <v>1102075</v>
+        <v/>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="7">
@@ -918,28 +918,28 @@
         <v>2026-10-12</v>
       </c>
       <c r="B7" t="str">
-        <v>A2610110770</v>
+        <v>A2610100732</v>
       </c>
       <c r="C7" t="str">
-        <v>SiCepat Ekspres Bogor Gunung Putri FM</v>
+        <v>SiCepat Ekspres Cikarang Utara FM</v>
       </c>
       <c r="D7" t="str">
-        <v>1223002</v>
+        <v>1209094</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
         <v>0</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J7" t="str">
         <v>12 OKT</v>
@@ -950,28 +950,28 @@
         <v>2026-10-12</v>
       </c>
       <c r="B8" t="str">
-        <v>A2610110773</v>
+        <v>A2610110733</v>
       </c>
       <c r="C8" t="str">
-        <v>SiCepat Ekspres Denpasar Barat FM</v>
+        <v>SiCepat Ekspres Jakut Penjaringan 2 FM</v>
       </c>
       <c r="D8" t="str">
-        <v>1701031</v>
+        <v>1102075</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8">
         <v>0</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" t="str">
         <v>12 OKT</v>
@@ -982,13 +982,13 @@
         <v>2026-10-12</v>
       </c>
       <c r="B9" t="str">
-        <v>A2610110812</v>
+        <v>A2610110770</v>
       </c>
       <c r="C9" t="str">
-        <v>SiCepat Ekspres Jakbar Cengkareng 2 FM</v>
+        <v>SiCepat Ekspres Bogor Gunung Putri FM</v>
       </c>
       <c r="D9" t="str">
-        <v>1103006</v>
+        <v>1223002</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -997,16 +997,16 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="J9" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="10">
@@ -1014,13 +1014,13 @@
         <v>2026-10-12</v>
       </c>
       <c r="B10" t="str">
-        <v>A2610120806</v>
+        <v>A2610110773</v>
       </c>
       <c r="C10" t="str">
-        <v>SiCepat Ekspres Jakbar Implant Kedoya</v>
+        <v>SiCepat Ekspres Denpasar Barat FM</v>
       </c>
       <c r="D10" t="str">
-        <v>1103011</v>
+        <v>1701031</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -1046,31 +1046,31 @@
         <v>2026-10-12</v>
       </c>
       <c r="B11" t="str">
-        <v>A2610120808</v>
+        <v>A2610110812</v>
       </c>
       <c r="C11" t="str">
-        <v>SiCepat Ekspres Bojonegoro Baureno</v>
+        <v>SiCepat Ekspres Jakbar Cengkareng 2 FM</v>
       </c>
       <c r="D11" t="str">
-        <v>T1614011</v>
+        <v>1103006</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="J11" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="12">
@@ -1078,13 +1078,13 @@
         <v>2026-10-12</v>
       </c>
       <c r="B12" t="str">
-        <v>A2610120813</v>
+        <v>A2610120806</v>
       </c>
       <c r="C12" t="str">
-        <v>SiCepat Ekspres Jakbar Kebon Jeruk FM</v>
+        <v>SiCepat Ekspres Jakbar Implant Kedoya</v>
       </c>
       <c r="D12" t="str">
-        <v>1103069</v>
+        <v>1103011</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -1093,16 +1093,16 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="J12" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="13">
@@ -1110,22 +1110,22 @@
         <v>2026-10-12</v>
       </c>
       <c r="B13" t="str">
-        <v>A2610120825</v>
+        <v>A2610120808</v>
       </c>
       <c r="C13" t="str">
-        <v>SiCepat Ekspres Jaktim Cakung 2 FM</v>
+        <v>SiCepat Ekspres Bojonegoro Baureno</v>
       </c>
       <c r="D13" t="str">
-        <v>1105064</v>
+        <v>T1614011</v>
       </c>
       <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
         <v>2</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>0</v>
-      </c>
-      <c r="G13">
-        <v>2</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -1134,7 +1134,7 @@
         <v>2</v>
       </c>
       <c r="J13" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="14">
@@ -1142,60 +1142,60 @@
         <v>2026-10-12</v>
       </c>
       <c r="B14" t="str">
-        <v>A2610120826</v>
+        <v>A2610120813</v>
       </c>
       <c r="C14" t="str">
-        <v>SiCepat Ekspres Jakarta Sortation</v>
+        <v>SiCepat Ekspres Jakbar Kebon Jeruk FM</v>
       </c>
       <c r="D14" t="str">
-        <v>1105056</v>
+        <v>1103069</v>
       </c>
       <c r="E14">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
       <c r="G14">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="H14">
         <v>0</v>
       </c>
       <c r="I14">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="J14" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B15" t="str">
-        <v>A2609302102</v>
+        <v>A2610120825</v>
       </c>
       <c r="C15" t="str">
-        <v>SiCepat Ekspres Batam Sortation</v>
+        <v>SiCepat Ekspres Jaktim Cakung 2 FM</v>
       </c>
       <c r="D15" t="str">
-        <v>502004</v>
+        <v>1105064</v>
       </c>
       <c r="E15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F15">
         <v>0</v>
       </c>
       <c r="G15">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="H15">
         <v>0</v>
       </c>
       <c r="I15">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="J15" t="str">
         <v>13 OKT</v>
@@ -1203,34 +1203,34 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B16" t="str">
-        <v>A2610080540</v>
+        <v>A2610120826</v>
       </c>
       <c r="C16" t="str">
-        <v>SiCepat Ekspres Demak LM</v>
+        <v>SiCepat Ekspres Jakarta Sortation</v>
       </c>
       <c r="D16" t="str">
-        <v>1420006</v>
+        <v>1105056</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H16">
         <v>0</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J16" t="str">
-        <v>14 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="17">
@@ -1238,19 +1238,19 @@
         <v>2026-10-13</v>
       </c>
       <c r="B17" t="str">
-        <v>A2610080552</v>
+        <v>A2610080540</v>
       </c>
       <c r="C17" t="str">
-        <v>Jakbar Kalideres FM</v>
+        <v>SiCepat Ekspres Demak LM</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>1420006</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -1259,10 +1259,10 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J17" t="str">
-        <v>13 OKT</v>
+        <v>14 OKT</v>
       </c>
     </row>
     <row r="18">
@@ -2565,55 +2565,55 @@
         <v>2026-10-12</v>
       </c>
       <c r="B3" t="str">
-        <v>A2610050285</v>
+        <v>A2609302102</v>
       </c>
       <c r="C3" t="str">
-        <v>SiCepat Ekspres Medan Sortation</v>
+        <v>SiCepat Ekspres Batam Sortation</v>
       </c>
       <c r="D3" t="str">
-        <v>201025</v>
+        <v>502004</v>
       </c>
       <c r="E3" t="str">
-        <v>SCANNER WIRELESS</v>
+        <v>KEYBOARD</v>
       </c>
       <c r="F3" t="str">
-        <v>ASSET BARU</v>
+        <v>ASSET RETUR</v>
       </c>
       <c r="G3" t="str">
         <v>TERKIRIM</v>
       </c>
       <c r="H3">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I3">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K3">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L3" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M3" t="str">
-        <v>39460; 39960; 40260; 41560; 38124; 36285; 41660; 35884; 41460; 36185</v>
+        <v>202410003040; A1100105429; A0800067072; A0700003625; A0800045977; 20232039737</v>
       </c>
       <c r="N3" t="str">
-        <v>999006709744</v>
+        <v/>
       </c>
       <c r="O3" t="str">
-        <v>CS22036216612; CS22036216632; CS22036216629; CS22036216633; CS22036216625; CS22036216627; CS22036216626; CS22036216622; CS22036216620; CS22036216630</v>
+        <v>2101SC33JZD8; 2050SC33LAB8; 2127SC31AD48; 2050SC33G6J8; 2010SC302EQ8; 2032SC32FXN8</v>
       </c>
       <c r="P3" t="str">
         <v/>
       </c>
       <c r="Q3" t="str">
-        <v>PERGANTIAN</v>
+        <v>PENAMBAHAN</v>
       </c>
       <c r="R3" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="4">
@@ -2621,19 +2621,19 @@
         <v>2026-10-12</v>
       </c>
       <c r="B4" t="str">
-        <v>A2610080518</v>
+        <v>A2609302102</v>
       </c>
       <c r="C4" t="str">
-        <v>SiCepat Ekspres Jombang Sortation</v>
+        <v>SiCepat Ekspres Batam Sortation</v>
       </c>
       <c r="D4" t="str">
-        <v>1618003</v>
+        <v>502004</v>
       </c>
       <c r="E4" t="str">
-        <v>SCANNER WIRELESS</v>
+        <v>KOMPUTER RAKITAN</v>
       </c>
       <c r="F4" t="str">
-        <v>ASSET BARU</v>
+        <v>ASSET RETUR</v>
       </c>
       <c r="G4" t="str">
         <v>TERKIRIM</v>
@@ -2654,13 +2654,13 @@
         <v>qty-kolom</v>
       </c>
       <c r="M4" t="str">
-        <v>39660; 35985; 37924; 39560; 39760; 40160</v>
+        <v>A130026153; A130026211; A130026187; A130026192; A130026151; A130026159</v>
       </c>
       <c r="N4" t="str">
-        <v>999006709778</v>
+        <v>999006724979; 999006724994; 999006725002; 999006725013; 999006725037; 999006725047</v>
       </c>
       <c r="O4" t="str">
-        <v>CS22036216621; CS22036216613; CS22036219817; CS22036219830; CS22036219823; CS22036219813</v>
+        <v>V3165SB380260600486; V3165SB380260700469; V3165SB380260700130; V3165SB380260700404; V3165SB380251200961; V3165SB380260701391</v>
       </c>
       <c r="P4" t="str">
         <v/>
@@ -2669,7 +2669,7 @@
         <v>PENAMBAHAN</v>
       </c>
       <c r="R4" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="5">
@@ -2677,55 +2677,55 @@
         <v>2026-10-12</v>
       </c>
       <c r="B5" t="str">
-        <v>A2610100732</v>
+        <v>A2609302102</v>
       </c>
       <c r="C5" t="str">
-        <v>SiCepat Ekspres Cikarang Utara FM</v>
+        <v>SiCepat Ekspres Batam Sortation</v>
       </c>
       <c r="D5" t="str">
-        <v>1209094</v>
+        <v>502004</v>
       </c>
       <c r="E5" t="str">
-        <v>SCANNER WIRELESS</v>
+        <v>MONITOR</v>
       </c>
       <c r="F5" t="str">
-        <v>ASSET BARU</v>
+        <v>ASSET RETUR</v>
       </c>
       <c r="G5" t="str">
         <v>TERKIRIM</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L5" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M5" t="str">
-        <v>40263; 39663; 36088; 38127; 41462</v>
+        <v>A1300027473; 55859; 20232000609; A0700002706; A0800032471; A0500001498</v>
       </c>
       <c r="N5" t="str">
-        <v>999006709809</v>
+        <v>999006725081; 999006725091; 999006725099; 999006725108; 999006725116; 999006725129</v>
       </c>
       <c r="O5" t="str">
-        <v>CS22036216628; CS22036216635; CS22036216611; CS22036216610; CS22036216616</v>
+        <v>1CR0040YP3; 1CR9201JXV; 1CR8320YQR; 1CR8320K1W; 1CR847038V; 1CR9201J51</v>
       </c>
       <c r="P5" t="str">
         <v/>
       </c>
       <c r="Q5" t="str">
-        <v>PERGANTIAN</v>
+        <v>PENAMBAHAN</v>
       </c>
       <c r="R5" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="6">
@@ -2733,55 +2733,55 @@
         <v>2026-10-12</v>
       </c>
       <c r="B6" t="str">
-        <v>A2610110733</v>
+        <v>A2609302102</v>
       </c>
       <c r="C6" t="str">
-        <v>SiCepat Ekspres Jakut Penjaringan 2 FM</v>
+        <v>SiCepat Ekspres Batam Sortation</v>
       </c>
       <c r="D6" t="str">
-        <v>1102075</v>
+        <v>502004</v>
       </c>
       <c r="E6" t="str">
-        <v>DVR 32 Ch</v>
+        <v>MOUSE</v>
       </c>
       <c r="F6" t="str">
-        <v>ASSET BARU</v>
+        <v>ASSET RETUR</v>
       </c>
       <c r="G6" t="str">
         <v>TERKIRIM</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L6" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M6" t="str">
-        <v>115581</v>
+        <v>A1600010652; A1100011138; A0700012758; A1100012130; 202610005688; A0800152241</v>
       </c>
       <c r="N6" t="str">
-        <v>999006709822</v>
+        <v/>
       </c>
       <c r="O6" t="str">
-        <v>GH1100373</v>
+        <v>SUDAH; SUDAH; SUDAH; SUDAH; SUDAH; SUDAH</v>
       </c>
       <c r="P6" t="str">
         <v/>
       </c>
       <c r="Q6" t="str">
-        <v>PERGANTIAN</v>
+        <v>PENAMBAHAN</v>
       </c>
       <c r="R6" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="7">
@@ -2789,16 +2789,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B7" t="str">
-        <v>A2610110733</v>
+        <v>A2610050285</v>
       </c>
       <c r="C7" t="str">
-        <v>SiCepat Ekspres Jakut Penjaringan 2 FM</v>
+        <v>SiCepat Ekspres Medan Sortation</v>
       </c>
       <c r="D7" t="str">
-        <v>1102075</v>
+        <v>201025</v>
       </c>
       <c r="E7" t="str">
-        <v>HARDISK 4 TB</v>
+        <v>SCANNER WIRELESS</v>
       </c>
       <c r="F7" t="str">
         <v>ASSET BARU</v>
@@ -2807,34 +2807,34 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L7" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M7" t="str">
-        <v>SUDAH</v>
+        <v>39460; 39960; 40260; 41560; 38124; 36285; 41660; 35884; 41460; 36185</v>
       </c>
       <c r="N7" t="str">
-        <v/>
+        <v>999006709744</v>
       </c>
       <c r="O7" t="str">
-        <v>SUDAH</v>
+        <v>CS22036216612; CS22036216632; CS22036216629; CS22036216633; CS22036216625; CS22036216627; CS22036216626; CS22036216622; CS22036216620; CS22036216630</v>
       </c>
       <c r="P7" t="str">
         <v/>
       </c>
       <c r="Q7" t="str">
-        <v/>
+        <v>PERGANTIAN</v>
       </c>
       <c r="R7" t="str">
         <v>12 OKT</v>
@@ -2845,52 +2845,52 @@
         <v>2026-10-12</v>
       </c>
       <c r="B8" t="str">
-        <v>A2610110770</v>
+        <v>A2610080518</v>
       </c>
       <c r="C8" t="str">
-        <v>SiCepat Ekspres Bogor Gunung Putri FM</v>
+        <v>SiCepat Ekspres Jombang Sortation</v>
       </c>
       <c r="D8" t="str">
-        <v>1223002</v>
+        <v>1618003</v>
       </c>
       <c r="E8" t="str">
-        <v>CPU RAKITAN</v>
+        <v>SCANNER WIRELESS</v>
       </c>
       <c r="F8" t="str">
-        <v>ASSET RETUR</v>
+        <v>ASSET BARU</v>
       </c>
       <c r="G8" t="str">
         <v>TERKIRIM</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L8" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M8" t="str">
-        <v>A130026162</v>
+        <v>39660; 35985; 37924; 39560; 39760; 40160</v>
       </c>
       <c r="N8" t="str">
-        <v>999006709844</v>
+        <v>999006709778</v>
       </c>
       <c r="O8" t="str">
-        <v>V3165SB380260601375</v>
+        <v>CS22036216621; CS22036216613; CS22036219817; CS22036219830; CS22036219823; CS22036219813</v>
       </c>
       <c r="P8" t="str">
         <v/>
       </c>
       <c r="Q8" t="str">
-        <v>PERGANTIAN</v>
+        <v>PENAMBAHAN</v>
       </c>
       <c r="R8" t="str">
         <v>12 OKT</v>
@@ -2901,16 +2901,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B9" t="str">
-        <v>A2610110773</v>
+        <v>A2610080552</v>
       </c>
       <c r="C9" t="str">
-        <v>SiCepat Ekspres Denpasar Barat FM</v>
+        <v>Jakbar Kalideres FM</v>
       </c>
       <c r="D9" t="str">
-        <v>1701031</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>PRINTER TSC</v>
+        <v>LAPTOP CORE I3</v>
       </c>
       <c r="F9" t="str">
         <v>ASSET RETUR</v>
@@ -2934,22 +2934,22 @@
         <v>qty-kolom</v>
       </c>
       <c r="M9" t="str">
-        <v>5548</v>
+        <v>202610007275</v>
       </c>
       <c r="N9" t="str">
-        <v>999006709868</v>
+        <v>999006726296</v>
       </c>
       <c r="O9" t="str">
-        <v>24P22024514</v>
+        <v>PF2JJNF5</v>
       </c>
       <c r="P9" t="str">
         <v/>
       </c>
       <c r="Q9" t="str">
-        <v>PERGANTIAN</v>
+        <v/>
       </c>
       <c r="R9" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="10">
@@ -2957,55 +2957,55 @@
         <v>2026-10-12</v>
       </c>
       <c r="B10" t="str">
-        <v>A2610110812</v>
+        <v>A2610100732</v>
       </c>
       <c r="C10" t="str">
-        <v>SiCepat Ekspres Jakbar Cengkareng 2 FM</v>
+        <v>SiCepat Ekspres Cikarang Utara FM</v>
       </c>
       <c r="D10" t="str">
-        <v>1103006</v>
+        <v>1209094</v>
       </c>
       <c r="E10" t="str">
-        <v>SCANNER KABEL 2D</v>
+        <v>SCANNER WIRELESS</v>
       </c>
       <c r="F10" t="str">
-        <v>ASSET RETUR</v>
+        <v>ASSET BARU</v>
       </c>
       <c r="G10" t="str">
         <v>TERKIRIM</v>
       </c>
       <c r="H10">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I10">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="J10">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="K10">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="L10" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M10" t="str">
-        <v>A0900010838; A0900013979; 20232020074; A0500003672; A1100037051; A1100120012; 202610002414; A1100113139; A0900014939; A0800191969; A1100034390; A1000005058; A0900013158; A0700084499</v>
+        <v>40263; 39663; 36088; 38127; 41462</v>
       </c>
       <c r="N10" t="str">
-        <v>999006724876</v>
+        <v>999006709809</v>
       </c>
       <c r="O10" t="str">
-        <v>TANPA SN; 21051B17445; 5J202009197; 21091B18257; TANPA SN; TANPA SN; 21051B17392; 21043B16331; 21121B7439; 5J202010249; 21051B17067; TANPA SN; 21051B17925; TANPA SN</v>
+        <v>CS22036216628; CS22036216635; CS22036216611; CS22036216610; CS22036216616</v>
       </c>
       <c r="P10" t="str">
         <v/>
       </c>
       <c r="Q10" t="str">
-        <v/>
+        <v>PERGANTIAN</v>
       </c>
       <c r="R10" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="11">
@@ -3013,19 +3013,19 @@
         <v>2026-10-12</v>
       </c>
       <c r="B11" t="str">
-        <v>A2610120806</v>
+        <v>A2610110733</v>
       </c>
       <c r="C11" t="str">
-        <v>SiCepat Ekspres Jakbar Implant Kedoya</v>
+        <v>SiCepat Ekspres Jakut Penjaringan 2 FM</v>
       </c>
       <c r="D11" t="str">
-        <v>1103011</v>
+        <v>1102075</v>
       </c>
       <c r="E11" t="str">
-        <v>SCANNER WIRELESS</v>
+        <v>DVR 32 Ch</v>
       </c>
       <c r="F11" t="str">
-        <v>ASSET RETUR</v>
+        <v>ASSET BARU</v>
       </c>
       <c r="G11" t="str">
         <v>TERKIRIM</v>
@@ -3046,13 +3046,13 @@
         <v>qty-kolom</v>
       </c>
       <c r="M11" t="str">
-        <v>40360</v>
+        <v>115581</v>
       </c>
       <c r="N11" t="str">
-        <v>999006709888</v>
+        <v>999006709822</v>
       </c>
       <c r="O11" t="str">
-        <v>CS2203226343</v>
+        <v>GH1100373</v>
       </c>
       <c r="P11" t="str">
         <v/>
@@ -3069,16 +3069,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B12" t="str">
-        <v>A2610120808</v>
+        <v>A2610110733</v>
       </c>
       <c r="C12" t="str">
-        <v>SiCepat Ekspres Bojonegoro Baureno</v>
+        <v>SiCepat Ekspres Jakut Penjaringan 2 FM</v>
       </c>
       <c r="D12" t="str">
-        <v>T1614011</v>
+        <v>1102075</v>
       </c>
       <c r="E12" t="str">
-        <v>SCANNER WIRELESS</v>
+        <v>HARDISK 4 TB</v>
       </c>
       <c r="F12" t="str">
         <v>ASSET BARU</v>
@@ -3087,34 +3087,34 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L12" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M12" t="str">
-        <v>38024; 35784</v>
+        <v>SUDAH</v>
       </c>
       <c r="N12" t="str">
-        <v>999006709932</v>
+        <v/>
       </c>
       <c r="O12" t="str">
-        <v>CS22036216623; CS22036216606</v>
+        <v>SUDAH</v>
       </c>
       <c r="P12" t="str">
         <v/>
       </c>
       <c r="Q12" t="str">
-        <v>PERGANTIAN</v>
+        <v/>
       </c>
       <c r="R12" t="str">
         <v>12 OKT</v>
@@ -3125,16 +3125,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B13" t="str">
-        <v>A2610120813</v>
+        <v>A2610110770</v>
       </c>
       <c r="C13" t="str">
-        <v>SiCepat Ekspres Jakbar Kebon Jeruk FM</v>
+        <v>SiCepat Ekspres Bogor Gunung Putri FM</v>
       </c>
       <c r="D13" t="str">
-        <v>1103069</v>
+        <v>1223002</v>
       </c>
       <c r="E13" t="str">
-        <v>SCANNER KABEL 2D</v>
+        <v>CPU RAKITAN</v>
       </c>
       <c r="F13" t="str">
         <v>ASSET RETUR</v>
@@ -3143,37 +3143,37 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H13">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="I13">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="J13">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="K13">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="L13" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M13" t="str">
-        <v>A0800043358; A0800200933; A1000003737; A130026817; A0900016481; A0700086666; A1100035327; 202610004956; A0900011158; A0900011155; A0900014483; 19597; A1100113771; A1100030250; A0500003273; A0900010591; A1100112420; A130024548; A1100034365; A1000003120; A1100112323; A0800051094; A0900014462; A130026834; A0800018454; A1100043214; A1100030973; A0700097464; A1100009082; A1100115203</v>
+        <v>A130026162</v>
       </c>
       <c r="N13" t="str">
-        <v>999006724934</v>
+        <v>999006709844</v>
       </c>
       <c r="O13" t="str">
-        <v>21043B16464; 21051B16080; TANPA SN; 21091B18159; 21043B16447; TANPA SN; TANPA SN; TANPA SN; 21051B17366; TANPA SN; TANPA SN; TANPA SN; TANPA SN; TANPA SN; 5J2020120025; 5J202010279; 21122B8274; 5J2020120028; 21051B17057; 21122B8271; TANPA SN; TANPA SN; 5J2020120080; TANPA SN; 3J6019020302; 5J2021010841; TANPA SN; TANPA SN; 21043B16334; TANPA SN</v>
+        <v>V3165SB380260601375</v>
       </c>
       <c r="P13" t="str">
         <v/>
       </c>
       <c r="Q13" t="str">
-        <v/>
+        <v>PERGANTIAN</v>
       </c>
       <c r="R13" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="14">
@@ -3181,16 +3181,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B14" t="str">
-        <v>A2610120825</v>
+        <v>A2610110773</v>
       </c>
       <c r="C14" t="str">
-        <v>SiCepat Ekspres Jaktim Cakung 2 FM</v>
+        <v>SiCepat Ekspres Denpasar Barat FM</v>
       </c>
       <c r="D14" t="str">
-        <v>1105064</v>
+        <v>1701031</v>
       </c>
       <c r="E14" t="str">
-        <v>RAK SERVER 6U</v>
+        <v>PRINTER TSC</v>
       </c>
       <c r="F14" t="str">
         <v>ASSET RETUR</v>
@@ -3214,22 +3214,22 @@
         <v>qty-kolom</v>
       </c>
       <c r="M14" t="str">
-        <v>A130025324</v>
+        <v>5548</v>
       </c>
       <c r="N14" t="str">
-        <v>SJ-054086</v>
+        <v>999006709868</v>
       </c>
       <c r="O14" t="str">
-        <v>P 60 CM L 45 CM T 37 CM</v>
+        <v>24P22024514</v>
       </c>
       <c r="P14" t="str">
         <v/>
       </c>
       <c r="Q14" t="str">
-        <v/>
+        <v>PERGANTIAN</v>
       </c>
       <c r="R14" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="15">
@@ -3237,16 +3237,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B15" t="str">
-        <v>A2610120825</v>
+        <v>A2610110812</v>
       </c>
       <c r="C15" t="str">
-        <v>SiCepat Ekspres Jaktim Cakung 2 FM</v>
+        <v>SiCepat Ekspres Jakbar Cengkareng 2 FM</v>
       </c>
       <c r="D15" t="str">
-        <v>1105064</v>
+        <v>1103006</v>
       </c>
       <c r="E15" t="str">
-        <v>RAK SERVER 8U</v>
+        <v>SCANNER KABEL 2D</v>
       </c>
       <c r="F15" t="str">
         <v>ASSET RETUR</v>
@@ -3255,28 +3255,28 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="K15">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="L15" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M15" t="str">
-        <v>A130026819</v>
+        <v>A0900010838; A0900013979; 20232020074; A0500003672; A1100037051; A1100120012; 202610002414; A1100113139; A0900014939; A0800191969; A1100034390; A1000005058; A0900013158; A0700084499</v>
       </c>
       <c r="N15" t="str">
-        <v>SJ-054086</v>
+        <v>999006724876</v>
       </c>
       <c r="O15" t="str">
-        <v>P 55 CM L 40 CM T45 CM</v>
+        <v>TANPA SN; 21051B17445; 5J202009197; 21091B18257; TANPA SN; TANPA SN; 21051B17392; 21043B16331; 21121B7439; 5J202010249; 21051B17067; TANPA SN; 21051B17925; TANPA SN</v>
       </c>
       <c r="P15" t="str">
         <v/>
@@ -3293,16 +3293,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B16" t="str">
-        <v>A2610120826</v>
+        <v>A2610120806</v>
       </c>
       <c r="C16" t="str">
-        <v>SiCepat Ekspres Jakarta Sortation</v>
+        <v>SiCepat Ekspres Jakbar Implant Kedoya</v>
       </c>
       <c r="D16" t="str">
-        <v>1105056</v>
+        <v>1103011</v>
       </c>
       <c r="E16" t="str">
-        <v>CAMERA IPEVO</v>
+        <v>SCANNER WIRELESS</v>
       </c>
       <c r="F16" t="str">
         <v>ASSET RETUR</v>
@@ -3326,19 +3326,19 @@
         <v>qty-kolom</v>
       </c>
       <c r="M16" t="str">
-        <v>A110050838</v>
+        <v>40360</v>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>999006709888</v>
       </c>
       <c r="O16" t="str">
-        <v>332022VAC01275</v>
+        <v>CS2203226343</v>
       </c>
       <c r="P16" t="str">
         <v/>
       </c>
       <c r="Q16" t="str">
-        <v/>
+        <v>PERGANTIAN</v>
       </c>
       <c r="R16" t="str">
         <v>12 OKT</v>
@@ -3349,52 +3349,52 @@
         <v>2026-10-12</v>
       </c>
       <c r="B17" t="str">
-        <v>A2610120826</v>
+        <v>A2610120808</v>
       </c>
       <c r="C17" t="str">
-        <v>SiCepat Ekspres Jakarta Sortation</v>
+        <v>SiCepat Ekspres Bojonegoro Baureno</v>
       </c>
       <c r="D17" t="str">
-        <v>1105056</v>
+        <v>T1614011</v>
       </c>
       <c r="E17" t="str">
-        <v>KEYBOARD KABEL</v>
+        <v>SCANNER WIRELESS</v>
       </c>
       <c r="F17" t="str">
-        <v>ASSET RETUR</v>
+        <v>ASSET BARU</v>
       </c>
       <c r="G17" t="str">
         <v>TERKIRIM</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L17" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M17" t="str">
-        <v>A0900014276</v>
+        <v>38024; 35784</v>
       </c>
       <c r="N17" t="str">
-        <v/>
+        <v>999006709932</v>
       </c>
       <c r="O17" t="str">
-        <v>2015SC31K1V8</v>
+        <v>CS22036216623; CS22036216606</v>
       </c>
       <c r="P17" t="str">
         <v/>
       </c>
       <c r="Q17" t="str">
-        <v/>
+        <v>PERGANTIAN</v>
       </c>
       <c r="R17" t="str">
         <v>12 OKT</v>
@@ -3405,16 +3405,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B18" t="str">
-        <v>A2610120826</v>
+        <v>A2610120813</v>
       </c>
       <c r="C18" t="str">
-        <v>SiCepat Ekspres Jakarta Sortation</v>
+        <v>SiCepat Ekspres Jakbar Kebon Jeruk FM</v>
       </c>
       <c r="D18" t="str">
-        <v>1105056</v>
+        <v>1103069</v>
       </c>
       <c r="E18" t="str">
-        <v>KOMPUTER RAKITAN</v>
+        <v>SCANNER KABEL 2D</v>
       </c>
       <c r="F18" t="str">
         <v>ASSET RETUR</v>
@@ -3423,28 +3423,28 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="J18">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="K18">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="L18" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M18" t="str">
-        <v>A130026196</v>
+        <v>A0800043358; A0800200933; A1000003737; A130026817; A0900016481; A0700086666; A1100035327; 202610004956; A0900011158; A0900011155; A0900014483; 19597; A1100113771; A1100030250; A0500003273; A0900010591; A1100112420; A130024548; A1100034365; A1000003120; A1100112323; A0800051094; A0900014462; A130026834; A0800018454; A1100043214; A1100030973; A0700097464; A1100009082; A1100115203</v>
       </c>
       <c r="N18" t="str">
-        <v>DIKIRIM DRIVER BESOK</v>
+        <v>999006724934</v>
       </c>
       <c r="O18" t="str">
-        <v>V3165SB380260700825</v>
+        <v>21043B16464; 21051B16080; TANPA SN; 21091B18159; 21043B16447; TANPA SN; TANPA SN; TANPA SN; 21051B17366; TANPA SN; TANPA SN; TANPA SN; TANPA SN; TANPA SN; 5J2020120025; 5J202010279; 21122B8274; 5J2020120028; 21051B17057; 21122B8271; TANPA SN; TANPA SN; 5J2020120080; TANPA SN; 3J6019020302; 5J2021010841; TANPA SN; TANPA SN; 21043B16334; TANPA SN</v>
       </c>
       <c r="P18" t="str">
         <v/>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="R18" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="19">
@@ -3461,16 +3461,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B19" t="str">
-        <v>A2610120826</v>
+        <v>A2610120825</v>
       </c>
       <c r="C19" t="str">
-        <v>SiCepat Ekspres Jakarta Sortation</v>
+        <v>SiCepat Ekspres Jaktim Cakung 2 FM</v>
       </c>
       <c r="D19" t="str">
-        <v>1105056</v>
+        <v>1105064</v>
       </c>
       <c r="E19" t="str">
-        <v>MONITOR SET</v>
+        <v>RAK SERVER 6U</v>
       </c>
       <c r="F19" t="str">
         <v>ASSET RETUR</v>
@@ -3494,22 +3494,22 @@
         <v>qty-kolom</v>
       </c>
       <c r="M19" t="str">
-        <v>20232036655</v>
+        <v>A130025324</v>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>SJ-054086</v>
       </c>
       <c r="O19" t="str">
-        <v>1CR00304S2</v>
+        <v>P 60 CM L 45 CM T 37 CM</v>
       </c>
       <c r="P19" t="str">
-        <v>HP V190</v>
+        <v/>
       </c>
       <c r="Q19" t="str">
         <v/>
       </c>
       <c r="R19" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="20">
@@ -3517,16 +3517,16 @@
         <v>2026-10-12</v>
       </c>
       <c r="B20" t="str">
-        <v>A2610120826</v>
+        <v>A2610120825</v>
       </c>
       <c r="C20" t="str">
-        <v>SiCepat Ekspres Jakarta Sortation</v>
+        <v>SiCepat Ekspres Jaktim Cakung 2 FM</v>
       </c>
       <c r="D20" t="str">
-        <v>1105056</v>
+        <v>1105064</v>
       </c>
       <c r="E20" t="str">
-        <v>PRINTER TSC</v>
+        <v>RAK SERVER 8U</v>
       </c>
       <c r="F20" t="str">
         <v>ASSET RETUR</v>
@@ -3550,13 +3550,13 @@
         <v>qty-kolom</v>
       </c>
       <c r="M20" t="str">
-        <v>96037</v>
+        <v>A130026819</v>
       </c>
       <c r="N20" t="str">
-        <v/>
+        <v>SJ-054086</v>
       </c>
       <c r="O20" t="str">
-        <v>24P25101257</v>
+        <v>P 55 CM L 40 CM T45 CM</v>
       </c>
       <c r="P20" t="str">
         <v/>
@@ -3565,7 +3565,7 @@
         <v/>
       </c>
       <c r="R20" t="str">
-        <v>12 OKT</v>
+        <v>13 OKT</v>
       </c>
     </row>
     <row r="21">
@@ -3582,7 +3582,7 @@
         <v>1105056</v>
       </c>
       <c r="E21" t="str">
-        <v>SCANNER WIRELESS</v>
+        <v>CAMERA IPEVO</v>
       </c>
       <c r="F21" t="str">
         <v>ASSET RETUR</v>
@@ -3606,13 +3606,13 @@
         <v>qty-kolom</v>
       </c>
       <c r="M21" t="str">
-        <v>37923</v>
+        <v>A110050838</v>
       </c>
       <c r="N21" t="str">
         <v/>
       </c>
       <c r="O21" t="str">
-        <v>CS2203226749</v>
+        <v>332022VAC01275</v>
       </c>
       <c r="P21" t="str">
         <v/>
@@ -3638,7 +3638,7 @@
         <v>1105056</v>
       </c>
       <c r="E22" t="str">
-        <v>TIMBANGAN TOLEDO + KABEL</v>
+        <v>KEYBOARD KABEL</v>
       </c>
       <c r="F22" t="str">
         <v>ASSET RETUR</v>
@@ -3662,13 +3662,13 @@
         <v>qty-kolom</v>
       </c>
       <c r="M22" t="str">
-        <v>20232039722</v>
+        <v>A0900014276</v>
       </c>
       <c r="N22" t="str">
         <v/>
       </c>
       <c r="O22" t="str">
-        <v>C048602263</v>
+        <v>2015SC31K1V8</v>
       </c>
       <c r="P22" t="str">
         <v/>
@@ -3682,19 +3682,19 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B23" t="str">
-        <v>A2609302102</v>
+        <v>A2610120826</v>
       </c>
       <c r="C23" t="str">
-        <v>SiCepat Ekspres Batam Sortation</v>
+        <v>SiCepat Ekspres Jakarta Sortation</v>
       </c>
       <c r="D23" t="str">
-        <v>502004</v>
+        <v>1105056</v>
       </c>
       <c r="E23" t="str">
-        <v>KEYBOARD</v>
+        <v>KOMPUTER RAKITAN</v>
       </c>
       <c r="F23" t="str">
         <v>ASSET RETUR</v>
@@ -3703,54 +3703,54 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H23">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I23">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K23">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L23" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M23" t="str">
-        <v>202410003040; A1100105429; A0800067072; A0700003625; A0800045977; 20232039737</v>
+        <v>A130026196</v>
       </c>
       <c r="N23" t="str">
-        <v/>
+        <v>DIKIRIM DRIVER BESOK</v>
       </c>
       <c r="O23" t="str">
-        <v>2101SC33JZD8; 2050SC33LAB8; 2127SC31AD48; 2050SC33G6J8; 2010SC302EQ8; 2032SC32FXN8</v>
+        <v>V3165SB380260700825</v>
       </c>
       <c r="P23" t="str">
         <v/>
       </c>
       <c r="Q23" t="str">
-        <v>PENAMBAHAN</v>
+        <v/>
       </c>
       <c r="R23" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B24" t="str">
-        <v>A2609302102</v>
+        <v>A2610120826</v>
       </c>
       <c r="C24" t="str">
-        <v>SiCepat Ekspres Batam Sortation</v>
+        <v>SiCepat Ekspres Jakarta Sortation</v>
       </c>
       <c r="D24" t="str">
-        <v>502004</v>
+        <v>1105056</v>
       </c>
       <c r="E24" t="str">
-        <v>KOMPUTER RAKITAN</v>
+        <v>MONITOR SET</v>
       </c>
       <c r="F24" t="str">
         <v>ASSET RETUR</v>
@@ -3759,54 +3759,54 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H24">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I24">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J24">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K24">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L24" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M24" t="str">
-        <v>A130026153; A130026211; A130026187; A130026192; A130026151; A130026159</v>
+        <v>20232036655</v>
       </c>
       <c r="N24" t="str">
-        <v>999006724979; 999006724994; 999006725002; 999006725013; 999006725037; 999006725047</v>
+        <v/>
       </c>
       <c r="O24" t="str">
-        <v>V3165SB380260600486; V3165SB380260700469; V3165SB380260700130; V3165SB380260700404; V3165SB380251200961; V3165SB380260701391</v>
+        <v>1CR00304S2</v>
       </c>
       <c r="P24" t="str">
-        <v/>
+        <v>HP V190</v>
       </c>
       <c r="Q24" t="str">
-        <v>PENAMBAHAN</v>
+        <v/>
       </c>
       <c r="R24" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B25" t="str">
-        <v>A2609302102</v>
+        <v>A2610120826</v>
       </c>
       <c r="C25" t="str">
-        <v>SiCepat Ekspres Batam Sortation</v>
+        <v>SiCepat Ekspres Jakarta Sortation</v>
       </c>
       <c r="D25" t="str">
-        <v>502004</v>
+        <v>1105056</v>
       </c>
       <c r="E25" t="str">
-        <v>MONITOR</v>
+        <v>PRINTER TSC</v>
       </c>
       <c r="F25" t="str">
         <v>ASSET RETUR</v>
@@ -3815,54 +3815,54 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L25" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M25" t="str">
-        <v>A1300027473; 55859; 20232000609; A0700002706; A0800032471; A0500001498</v>
+        <v>96037</v>
       </c>
       <c r="N25" t="str">
-        <v>999006725081; 999006725091; 999006725099; 999006725108; 999006725116; 999006725129</v>
+        <v/>
       </c>
       <c r="O25" t="str">
-        <v>1CR0040YP3; 1CR9201JXV; 1CR8320YQR; 1CR8320K1W; 1CR847038V; 1CR9201J51</v>
+        <v>24P25101257</v>
       </c>
       <c r="P25" t="str">
         <v/>
       </c>
       <c r="Q25" t="str">
-        <v>PENAMBAHAN</v>
+        <v/>
       </c>
       <c r="R25" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B26" t="str">
-        <v>A2609302102</v>
+        <v>A2610120826</v>
       </c>
       <c r="C26" t="str">
-        <v>SiCepat Ekspres Batam Sortation</v>
+        <v>SiCepat Ekspres Jakarta Sortation</v>
       </c>
       <c r="D26" t="str">
-        <v>502004</v>
+        <v>1105056</v>
       </c>
       <c r="E26" t="str">
-        <v>MOUSE</v>
+        <v>SCANNER WIRELESS</v>
       </c>
       <c r="F26" t="str">
         <v>ASSET RETUR</v>
@@ -3871,54 +3871,54 @@
         <v>TERKIRIM</v>
       </c>
       <c r="H26">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I26">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K26">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L26" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M26" t="str">
-        <v>A1600010652; A1100011138; A0700012758; A1100012130; 202610005688; A0800152241</v>
+        <v>37923</v>
       </c>
       <c r="N26" t="str">
         <v/>
       </c>
       <c r="O26" t="str">
-        <v>SUDAH; SUDAH; SUDAH; SUDAH; SUDAH; SUDAH</v>
+        <v>CS2203226749</v>
       </c>
       <c r="P26" t="str">
         <v/>
       </c>
       <c r="Q26" t="str">
-        <v>PENAMBAHAN</v>
+        <v/>
       </c>
       <c r="R26" t="str">
-        <v>13 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B27" t="str">
-        <v>A2610080540</v>
+        <v>A2610120826</v>
       </c>
       <c r="C27" t="str">
-        <v>SiCepat Ekspres Demak LM</v>
+        <v>SiCepat Ekspres Jakarta Sortation</v>
       </c>
       <c r="D27" t="str">
-        <v>1420006</v>
+        <v>1105056</v>
       </c>
       <c r="E27" t="str">
-        <v>PRINTER CANON LASERJET</v>
+        <v>TIMBANGAN TOLEDO + KABEL</v>
       </c>
       <c r="F27" t="str">
         <v>ASSET RETUR</v>
@@ -3942,22 +3942,22 @@
         <v>qty-kolom</v>
       </c>
       <c r="M27" t="str">
-        <v>A1300027867</v>
+        <v>20232039722</v>
       </c>
       <c r="N27" t="str">
-        <v>999006738290</v>
+        <v/>
       </c>
       <c r="O27" t="str">
-        <v>NQSA111830</v>
+        <v>C048602263</v>
       </c>
       <c r="P27" t="str">
         <v/>
       </c>
       <c r="Q27" t="str">
-        <v>PERGANTIAN</v>
+        <v/>
       </c>
       <c r="R27" t="str">
-        <v>14 OKT</v>
+        <v>12 OKT</v>
       </c>
     </row>
     <row r="28">
@@ -3974,37 +3974,37 @@
         <v>1420006</v>
       </c>
       <c r="E28" t="str">
-        <v>SCANNER WIRELESS</v>
+        <v>PRINTER CANON LASERJET</v>
       </c>
       <c r="F28" t="str">
-        <v>ASSET BARU</v>
+        <v>ASSET RETUR</v>
       </c>
       <c r="G28" t="str">
         <v>TERKIRIM</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L28" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M28" t="str">
-        <v>39559; 41559</v>
+        <v>A1300027867</v>
       </c>
       <c r="N28" t="str">
-        <v>999006738321</v>
+        <v>999006738290</v>
       </c>
       <c r="O28" t="str">
-        <v>CS22036219812; CS22036219827</v>
+        <v>NQSA111830</v>
       </c>
       <c r="P28" t="str">
         <v/>
@@ -4021,55 +4021,55 @@
         <v>2026-10-13</v>
       </c>
       <c r="B29" t="str">
-        <v>A2610080552</v>
+        <v>A2610080540</v>
       </c>
       <c r="C29" t="str">
-        <v>Jakbar Kalideres FM</v>
+        <v>SiCepat Ekspres Demak LM</v>
       </c>
       <c r="D29" t="str">
-        <v/>
+        <v>1420006</v>
       </c>
       <c r="E29" t="str">
-        <v>LAPTOP CORE I3</v>
+        <v>SCANNER WIRELESS</v>
       </c>
       <c r="F29" t="str">
-        <v>ASSET RETUR</v>
+        <v>ASSET BARU</v>
       </c>
       <c r="G29" t="str">
         <v>TERKIRIM</v>
       </c>
       <c r="H29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L29" t="str">
         <v>qty-kolom</v>
       </c>
       <c r="M29" t="str">
-        <v>202610007275</v>
+        <v>39559; 41559</v>
       </c>
       <c r="N29" t="str">
-        <v>999006726296</v>
+        <v>999006738321</v>
       </c>
       <c r="O29" t="str">
-        <v>PF2JJNF5</v>
+        <v>CS22036219812; CS22036219827</v>
       </c>
       <c r="P29" t="str">
         <v/>
       </c>
       <c r="Q29" t="str">
-        <v/>
+        <v>PERGANTIAN</v>
       </c>
       <c r="R29" t="str">
-        <v>13 OKT</v>
+        <v>14 OKT</v>
       </c>
     </row>
     <row r="30">
@@ -16108,7 +16108,7 @@
         <v>MASUK</v>
       </c>
       <c r="D128" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E128" t="str">
         <v>A2609302102</v>
@@ -16161,7 +16161,7 @@
         <v>MASUK</v>
       </c>
       <c r="D129" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E129" t="str">
         <v>A2609302102</v>
@@ -16214,7 +16214,7 @@
         <v>MASUK</v>
       </c>
       <c r="D130" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E130" t="str">
         <v>A2609302102</v>
@@ -16267,7 +16267,7 @@
         <v>MASUK</v>
       </c>
       <c r="D131" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E131" t="str">
         <v>A2609302102</v>
@@ -16320,7 +16320,7 @@
         <v>MASUK</v>
       </c>
       <c r="D132" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E132" t="str">
         <v>A2609302102</v>
@@ -16373,7 +16373,7 @@
         <v>MASUK</v>
       </c>
       <c r="D133" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E133" t="str">
         <v>A2609302102</v>
@@ -16426,7 +16426,7 @@
         <v>MASUK</v>
       </c>
       <c r="D134" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E134" t="str">
         <v>A2609302102</v>
@@ -16479,7 +16479,7 @@
         <v>MASUK</v>
       </c>
       <c r="D135" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E135" t="str">
         <v>A2609302102</v>
@@ -16532,7 +16532,7 @@
         <v>MASUK</v>
       </c>
       <c r="D136" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E136" t="str">
         <v>A2609302102</v>
@@ -16585,7 +16585,7 @@
         <v>MASUK</v>
       </c>
       <c r="D137" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E137" t="str">
         <v>A2609302102</v>
@@ -16638,7 +16638,7 @@
         <v>MASUK</v>
       </c>
       <c r="D138" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E138" t="str">
         <v>A2609302102</v>
@@ -16691,7 +16691,7 @@
         <v>MASUK</v>
       </c>
       <c r="D139" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E139" t="str">
         <v>A2609302102</v>
@@ -16744,7 +16744,7 @@
         <v>MASUK</v>
       </c>
       <c r="D140" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E140" t="str">
         <v>A2609302102</v>
@@ -16797,7 +16797,7 @@
         <v>MASUK</v>
       </c>
       <c r="D141" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E141" t="str">
         <v>A2609302102</v>
@@ -16850,7 +16850,7 @@
         <v>MASUK</v>
       </c>
       <c r="D142" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E142" t="str">
         <v>A2609302102</v>
@@ -16903,7 +16903,7 @@
         <v>MASUK</v>
       </c>
       <c r="D143" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E143" t="str">
         <v>A2609302102</v>
@@ -16956,7 +16956,7 @@
         <v>MASUK</v>
       </c>
       <c r="D144" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E144" t="str">
         <v>A2609302102</v>
@@ -17009,7 +17009,7 @@
         <v>MASUK</v>
       </c>
       <c r="D145" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E145" t="str">
         <v>A2609302102</v>
@@ -17062,7 +17062,7 @@
         <v>MASUK</v>
       </c>
       <c r="D146" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E146" t="str">
         <v>A2609302102</v>
@@ -17115,7 +17115,7 @@
         <v>MASUK</v>
       </c>
       <c r="D147" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E147" t="str">
         <v>A2609302102</v>
@@ -17168,7 +17168,7 @@
         <v>MASUK</v>
       </c>
       <c r="D148" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E148" t="str">
         <v>A2609302102</v>
@@ -17221,7 +17221,7 @@
         <v>MASUK</v>
       </c>
       <c r="D149" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E149" t="str">
         <v>A2609302102</v>
@@ -17274,7 +17274,7 @@
         <v>MASUK</v>
       </c>
       <c r="D150" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E150" t="str">
         <v>A2609302102</v>
@@ -17327,7 +17327,7 @@
         <v>MASUK</v>
       </c>
       <c r="D151" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E151" t="str">
         <v>A2609302102</v>
@@ -17380,7 +17380,7 @@
         <v>MASUK</v>
       </c>
       <c r="D152" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="E152" t="str">
         <v>A2610080552</v>
@@ -30594,7 +30594,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>25 baris kolom tanggalnya kosong -&gt; di file upload-ulang sudah diisi tanggal file (13 OKT). Baris: 93, 94, 95, 96, 97, 98, 99, 100, 101, 102, 103, 104, 105, 106, 107, 108, 109, 110, 111, 112, 113, 114, 115, 116, 117. Tanggal ini ASUMSI dari nama file/sheet karena kolom tanggal di sheet kosong — kalau tanggal kirim sebenarnya beda, ubah di file upload-ulang sebelum di-upload.</v>
+        <v>25 baris (A2609302102 Batam Sortation 24 baris + A2610080552 1 baris) kolom tanggalnya kosong di sheet. Di file upload-ulang diisi 12-Oct-26 (keputusan 19 Okt 2026): hasil cek Supabase menunjukkan di sistem lama tersimpan 2026-10-11 = tanggal sumber 12 Okt kena bug mundur 1 hari, dan urutan resi 999006724979-999006726296 berada di perbatasan resi tgl 12 ke 13.</v>
       </c>
     </row>
     <row r="8">

</xml_diff>